<commit_message>
feat: add GuestDashboard component and API models for user authentication refresh
- Created GuestDashboard component for guest access information.
- Added API model for successful user authentication refresh (usersAuthRefreshCreate200).
- Added API model for failed user authentication refresh (usersAuthRefreshCreate401).
- Added versioned API models for successful (v1UsersAuthRefreshCreate200) and failed (v1UsersAuthRefreshCreate401) user authentication refresh.
- Bugfixes
- Added docs
</commit_message>
<xml_diff>
--- a/docs/sample.xlsx
+++ b/docs/sample.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29426"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\eren\Desktop\codes\Python\Django\ses\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu\home\erenimo\projects\ses\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D01971E9-6C7A-42D2-88C2-EAF80601CE23}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AC505BC6-1EA2-4A48-905B-F7485F148EC9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -509,151 +509,151 @@
     <t>Project(%10)_0833AB</t>
   </si>
   <si>
-    <t>202500001</t>
-  </si>
-  <si>
-    <t>202500002</t>
-  </si>
-  <si>
-    <t>202500003</t>
-  </si>
-  <si>
-    <t>202500004</t>
-  </si>
-  <si>
-    <t>202500005</t>
-  </si>
-  <si>
-    <t>202500006</t>
-  </si>
-  <si>
-    <t>202500007</t>
-  </si>
-  <si>
-    <t>202500008</t>
-  </si>
-  <si>
-    <t>202500009</t>
-  </si>
-  <si>
-    <t>202500010</t>
-  </si>
-  <si>
-    <t>202500011</t>
-  </si>
-  <si>
-    <t>202500012</t>
-  </si>
-  <si>
-    <t>202500013</t>
-  </si>
-  <si>
-    <t>202500014</t>
-  </si>
-  <si>
-    <t>202500015</t>
-  </si>
-  <si>
-    <t>202500016</t>
-  </si>
-  <si>
-    <t>202500017</t>
-  </si>
-  <si>
-    <t>202500018</t>
-  </si>
-  <si>
-    <t>202500019</t>
-  </si>
-  <si>
-    <t>202500020</t>
-  </si>
-  <si>
-    <t>202500021</t>
-  </si>
-  <si>
-    <t>202500022</t>
-  </si>
-  <si>
-    <t>202500023</t>
-  </si>
-  <si>
-    <t>202500024</t>
-  </si>
-  <si>
-    <t>202500025</t>
-  </si>
-  <si>
-    <t>202500026</t>
-  </si>
-  <si>
-    <t>202500027</t>
-  </si>
-  <si>
-    <t>202500028</t>
-  </si>
-  <si>
-    <t>202500029</t>
-  </si>
-  <si>
-    <t>202500030</t>
-  </si>
-  <si>
-    <t>202500031</t>
-  </si>
-  <si>
-    <t>202500032</t>
-  </si>
-  <si>
-    <t>202500033</t>
-  </si>
-  <si>
-    <t>202500034</t>
-  </si>
-  <si>
-    <t>202500035</t>
-  </si>
-  <si>
-    <t>202500036</t>
-  </si>
-  <si>
-    <t>202500037</t>
-  </si>
-  <si>
-    <t>202500038</t>
-  </si>
-  <si>
-    <t>202500039</t>
-  </si>
-  <si>
-    <t>202500040</t>
-  </si>
-  <si>
-    <t>202500041</t>
-  </si>
-  <si>
-    <t>202500042</t>
-  </si>
-  <si>
-    <t>202500043</t>
-  </si>
-  <si>
-    <t>202500044</t>
-  </si>
-  <si>
-    <t>202500045</t>
-  </si>
-  <si>
-    <t>202500046</t>
-  </si>
-  <si>
-    <t>202500047</t>
-  </si>
-  <si>
-    <t>202500048</t>
-  </si>
-  <si>
-    <t>202500049</t>
+    <t>221400026</t>
+  </si>
+  <si>
+    <t>221400027</t>
+  </si>
+  <si>
+    <t>221400028</t>
+  </si>
+  <si>
+    <t>221400029</t>
+  </si>
+  <si>
+    <t>221400030</t>
+  </si>
+  <si>
+    <t>221400031</t>
+  </si>
+  <si>
+    <t>221400032</t>
+  </si>
+  <si>
+    <t>221400033</t>
+  </si>
+  <si>
+    <t>221400034</t>
+  </si>
+  <si>
+    <t>221400035</t>
+  </si>
+  <si>
+    <t>221400036</t>
+  </si>
+  <si>
+    <t>221400037</t>
+  </si>
+  <si>
+    <t>221400038</t>
+  </si>
+  <si>
+    <t>221400039</t>
+  </si>
+  <si>
+    <t>221400040</t>
+  </si>
+  <si>
+    <t>221400041</t>
+  </si>
+  <si>
+    <t>221400042</t>
+  </si>
+  <si>
+    <t>221400043</t>
+  </si>
+  <si>
+    <t>221400044</t>
+  </si>
+  <si>
+    <t>221400045</t>
+  </si>
+  <si>
+    <t>221400046</t>
+  </si>
+  <si>
+    <t>221400047</t>
+  </si>
+  <si>
+    <t>221400048</t>
+  </si>
+  <si>
+    <t>221400049</t>
+  </si>
+  <si>
+    <t>221400050</t>
+  </si>
+  <si>
+    <t>221400051</t>
+  </si>
+  <si>
+    <t>221400052</t>
+  </si>
+  <si>
+    <t>221400053</t>
+  </si>
+  <si>
+    <t>221400054</t>
+  </si>
+  <si>
+    <t>221400055</t>
+  </si>
+  <si>
+    <t>221400056</t>
+  </si>
+  <si>
+    <t>221400057</t>
+  </si>
+  <si>
+    <t>221400058</t>
+  </si>
+  <si>
+    <t>221400059</t>
+  </si>
+  <si>
+    <t>221400060</t>
+  </si>
+  <si>
+    <t>221400061</t>
+  </si>
+  <si>
+    <t>221400062</t>
+  </si>
+  <si>
+    <t>221400063</t>
+  </si>
+  <si>
+    <t>221400064</t>
+  </si>
+  <si>
+    <t>221400065</t>
+  </si>
+  <si>
+    <t>221400066</t>
+  </si>
+  <si>
+    <t>221400067</t>
+  </si>
+  <si>
+    <t>221400068</t>
+  </si>
+  <si>
+    <t>221400069</t>
+  </si>
+  <si>
+    <t>221400070</t>
+  </si>
+  <si>
+    <t>221400071</t>
+  </si>
+  <si>
+    <t>221400072</t>
+  </si>
+  <si>
+    <t>221400073</t>
+  </si>
+  <si>
+    <t>221400074</t>
   </si>
 </sst>
 </file>
@@ -2022,8 +2022,8 @@
         <v>7</v>
       </c>
       <c r="G2" s="9">
-        <f t="shared" ref="G2:I50" ca="1" si="0">TRUNC(60 + ((RAND()*100 - 0) * (100 - 60) / (100 - 0)))</f>
-        <v>68</v>
+        <f t="shared" ref="G2:H50" ca="1" si="0">TRUNC(60 + ((RAND()*100 - 0) * (100 - 60) / (100 - 0)))</f>
+        <v>67</v>
       </c>
       <c r="H2" s="9">
         <f ca="1">TRUNC(60 + ((RAND()*100 - 0) * (100 - 60) / (100 - 0)))</f>
@@ -2031,11 +2031,11 @@
       </c>
       <c r="I2" s="9">
         <f ca="1">TRUNC(30 + ((RAND()*100 - 0) * (60 - 30) / (100 - 0)))</f>
-        <v>40</v>
+        <v>32</v>
       </c>
       <c r="J2" s="9">
         <f ca="1">TRUNC(30 + ((RAND()*100 - 0) * (60 - 30) / (100 - 0)))</f>
-        <v>36</v>
+        <v>55</v>
       </c>
       <c r="K2" s="6"/>
     </row>
@@ -2060,19 +2060,19 @@
       </c>
       <c r="G3" s="9">
         <f t="shared" ca="1" si="0"/>
-        <v>90</v>
+        <v>74</v>
       </c>
       <c r="H3" s="9">
         <f t="shared" ca="1" si="0"/>
-        <v>63</v>
+        <v>73</v>
       </c>
       <c r="I3" s="9">
         <f t="shared" ref="I3:J50" ca="1" si="1">TRUNC(30 + ((RAND()*100 - 0) * (60 - 30) / (100 - 0)))</f>
-        <v>49</v>
+        <v>44</v>
       </c>
       <c r="J3" s="9">
         <f t="shared" ca="1" si="1"/>
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="K3" s="8"/>
     </row>
@@ -2097,19 +2097,19 @@
       </c>
       <c r="G4" s="9">
         <f t="shared" ca="1" si="0"/>
-        <v>68</v>
+        <v>82</v>
       </c>
       <c r="H4" s="9">
         <f t="shared" ca="1" si="0"/>
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="I4" s="9">
         <f t="shared" ca="1" si="1"/>
-        <v>47</v>
+        <v>58</v>
       </c>
       <c r="J4" s="9">
         <f t="shared" ca="1" si="1"/>
-        <v>39</v>
+        <v>53</v>
       </c>
       <c r="K4" s="8"/>
     </row>
@@ -2134,19 +2134,19 @@
       </c>
       <c r="G5" s="9">
         <f t="shared" ca="1" si="0"/>
-        <v>72</v>
+        <v>79</v>
       </c>
       <c r="H5" s="9">
         <f t="shared" ca="1" si="0"/>
-        <v>92</v>
+        <v>75</v>
       </c>
       <c r="I5" s="9">
         <f t="shared" ca="1" si="1"/>
-        <v>41</v>
+        <v>55</v>
       </c>
       <c r="J5" s="9">
         <f t="shared" ca="1" si="1"/>
-        <v>44</v>
+        <v>31</v>
       </c>
       <c r="K5" s="8"/>
     </row>
@@ -2171,19 +2171,19 @@
       </c>
       <c r="G6" s="9">
         <f t="shared" ca="1" si="0"/>
-        <v>75</v>
+        <v>96</v>
       </c>
       <c r="H6" s="9">
         <f t="shared" ca="1" si="0"/>
-        <v>60</v>
+        <v>81</v>
       </c>
       <c r="I6" s="9">
         <f t="shared" ca="1" si="1"/>
-        <v>32</v>
+        <v>40</v>
       </c>
       <c r="J6" s="9">
         <f t="shared" ca="1" si="1"/>
-        <v>46</v>
+        <v>56</v>
       </c>
       <c r="K6" s="8"/>
     </row>
@@ -2208,19 +2208,19 @@
       </c>
       <c r="G7" s="9">
         <f t="shared" ca="1" si="0"/>
-        <v>84</v>
+        <v>73</v>
       </c>
       <c r="H7" s="9">
         <f t="shared" ca="1" si="0"/>
-        <v>66</v>
+        <v>95</v>
       </c>
       <c r="I7" s="9">
         <f t="shared" ca="1" si="1"/>
-        <v>55</v>
+        <v>44</v>
       </c>
       <c r="J7" s="9">
         <f t="shared" ca="1" si="1"/>
-        <v>51</v>
+        <v>48</v>
       </c>
       <c r="K7" s="8"/>
     </row>
@@ -2245,19 +2245,19 @@
       </c>
       <c r="G8" s="9">
         <f t="shared" ca="1" si="0"/>
-        <v>92</v>
+        <v>98</v>
       </c>
       <c r="H8" s="9">
         <f t="shared" ca="1" si="0"/>
-        <v>87</v>
+        <v>75</v>
       </c>
       <c r="I8" s="9">
         <f t="shared" ca="1" si="1"/>
-        <v>43</v>
+        <v>36</v>
       </c>
       <c r="J8" s="9">
         <f t="shared" ca="1" si="1"/>
-        <v>42</v>
+        <v>33</v>
       </c>
       <c r="K8" s="8"/>
     </row>
@@ -2282,19 +2282,19 @@
       </c>
       <c r="G9" s="9">
         <f t="shared" ca="1" si="0"/>
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="H9" s="9">
         <f t="shared" ca="1" si="0"/>
-        <v>74</v>
+        <v>69</v>
       </c>
       <c r="I9" s="9">
         <f t="shared" ca="1" si="1"/>
-        <v>44</v>
+        <v>53</v>
       </c>
       <c r="J9" s="9">
         <f t="shared" ca="1" si="1"/>
-        <v>48</v>
+        <v>33</v>
       </c>
       <c r="K9" s="8"/>
     </row>
@@ -2319,19 +2319,19 @@
       </c>
       <c r="G10" s="9">
         <f t="shared" ca="1" si="0"/>
-        <v>68</v>
+        <v>60</v>
       </c>
       <c r="H10" s="9">
         <f t="shared" ca="1" si="0"/>
-        <v>79</v>
+        <v>92</v>
       </c>
       <c r="I10" s="9">
         <f t="shared" ca="1" si="1"/>
-        <v>43</v>
+        <v>34</v>
       </c>
       <c r="J10" s="9">
         <f t="shared" ca="1" si="1"/>
-        <v>52</v>
+        <v>41</v>
       </c>
       <c r="K10" s="8"/>
     </row>
@@ -2356,19 +2356,19 @@
       </c>
       <c r="G11" s="9">
         <f t="shared" ca="1" si="0"/>
-        <v>92</v>
+        <v>97</v>
       </c>
       <c r="H11" s="9">
         <f t="shared" ca="1" si="0"/>
-        <v>83</v>
+        <v>98</v>
       </c>
       <c r="I11" s="9">
         <f t="shared" ca="1" si="1"/>
-        <v>32</v>
+        <v>56</v>
       </c>
       <c r="J11" s="9">
         <f t="shared" ca="1" si="1"/>
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="K11" s="8"/>
     </row>
@@ -2393,19 +2393,19 @@
       </c>
       <c r="G12" s="9">
         <f t="shared" ca="1" si="0"/>
-        <v>72</v>
+        <v>81</v>
       </c>
       <c r="H12" s="9">
         <f t="shared" ca="1" si="0"/>
-        <v>60</v>
+        <v>68</v>
       </c>
       <c r="I12" s="9">
         <f t="shared" ca="1" si="1"/>
-        <v>48</v>
+        <v>40</v>
       </c>
       <c r="J12" s="9">
         <f t="shared" ca="1" si="1"/>
-        <v>34</v>
+        <v>47</v>
       </c>
       <c r="K12" s="8"/>
     </row>
@@ -2430,19 +2430,19 @@
       </c>
       <c r="G13" s="9">
         <f t="shared" ca="1" si="0"/>
-        <v>70</v>
+        <v>64</v>
       </c>
       <c r="H13" s="9">
         <f t="shared" ca="1" si="0"/>
-        <v>80</v>
+        <v>72</v>
       </c>
       <c r="I13" s="9">
         <f t="shared" ca="1" si="1"/>
-        <v>54</v>
+        <v>37</v>
       </c>
       <c r="J13" s="9">
         <f t="shared" ca="1" si="1"/>
-        <v>52</v>
+        <v>45</v>
       </c>
       <c r="K13" s="8"/>
     </row>
@@ -2467,19 +2467,19 @@
       </c>
       <c r="G14" s="9">
         <f t="shared" ca="1" si="0"/>
-        <v>98</v>
+        <v>66</v>
       </c>
       <c r="H14" s="9">
         <f t="shared" ca="1" si="0"/>
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="I14" s="9">
         <f t="shared" ca="1" si="1"/>
-        <v>54</v>
+        <v>43</v>
       </c>
       <c r="J14" s="9">
         <f t="shared" ca="1" si="1"/>
-        <v>32</v>
+        <v>45</v>
       </c>
       <c r="K14" s="8"/>
     </row>
@@ -2504,19 +2504,19 @@
       </c>
       <c r="G15" s="9">
         <f t="shared" ca="1" si="0"/>
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="H15" s="9">
         <f t="shared" ca="1" si="0"/>
-        <v>89</v>
+        <v>61</v>
       </c>
       <c r="I15" s="9">
         <f t="shared" ca="1" si="1"/>
-        <v>30</v>
+        <v>35</v>
       </c>
       <c r="J15" s="9">
         <f t="shared" ca="1" si="1"/>
-        <v>57</v>
+        <v>42</v>
       </c>
       <c r="K15" s="8"/>
     </row>
@@ -2541,19 +2541,19 @@
       </c>
       <c r="G16" s="9">
         <f t="shared" ca="1" si="0"/>
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="H16" s="9">
         <f t="shared" ca="1" si="0"/>
-        <v>91</v>
+        <v>64</v>
       </c>
       <c r="I16" s="9">
         <f t="shared" ca="1" si="1"/>
-        <v>43</v>
+        <v>32</v>
       </c>
       <c r="J16" s="9">
         <f t="shared" ca="1" si="1"/>
-        <v>31</v>
+        <v>59</v>
       </c>
       <c r="K16" s="8"/>
     </row>
@@ -2578,19 +2578,19 @@
       </c>
       <c r="G17" s="9">
         <f t="shared" ca="1" si="0"/>
-        <v>82</v>
+        <v>71</v>
       </c>
       <c r="H17" s="9">
         <f t="shared" ca="1" si="0"/>
-        <v>88</v>
+        <v>75</v>
       </c>
       <c r="I17" s="9">
         <f t="shared" ca="1" si="1"/>
-        <v>58</v>
+        <v>49</v>
       </c>
       <c r="J17" s="9">
         <f t="shared" ca="1" si="1"/>
-        <v>54</v>
+        <v>43</v>
       </c>
       <c r="K17" s="8"/>
     </row>
@@ -2615,19 +2615,19 @@
       </c>
       <c r="G18" s="9">
         <f t="shared" ca="1" si="0"/>
-        <v>85</v>
+        <v>82</v>
       </c>
       <c r="H18" s="9">
         <f t="shared" ca="1" si="0"/>
-        <v>85</v>
+        <v>96</v>
       </c>
       <c r="I18" s="9">
         <f t="shared" ca="1" si="1"/>
-        <v>40</v>
+        <v>54</v>
       </c>
       <c r="J18" s="9">
         <f t="shared" ca="1" si="1"/>
-        <v>30</v>
+        <v>36</v>
       </c>
       <c r="K18" s="8"/>
     </row>
@@ -2652,19 +2652,19 @@
       </c>
       <c r="G19" s="9">
         <f t="shared" ca="1" si="0"/>
-        <v>87</v>
+        <v>95</v>
       </c>
       <c r="H19" s="9">
         <f t="shared" ca="1" si="0"/>
-        <v>82</v>
+        <v>93</v>
       </c>
       <c r="I19" s="9">
         <f t="shared" ca="1" si="1"/>
-        <v>59</v>
+        <v>45</v>
       </c>
       <c r="J19" s="9">
         <f t="shared" ca="1" si="1"/>
-        <v>40</v>
+        <v>44</v>
       </c>
       <c r="K19" s="8"/>
     </row>
@@ -2689,19 +2689,19 @@
       </c>
       <c r="G20" s="9">
         <f t="shared" ca="1" si="0"/>
-        <v>64</v>
+        <v>89</v>
       </c>
       <c r="H20" s="9">
         <f t="shared" ca="1" si="0"/>
-        <v>77</v>
+        <v>67</v>
       </c>
       <c r="I20" s="9">
         <f t="shared" ca="1" si="1"/>
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="J20" s="9">
         <f t="shared" ca="1" si="1"/>
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="K20" s="8"/>
     </row>
@@ -2726,19 +2726,19 @@
       </c>
       <c r="G21" s="9">
         <f t="shared" ca="1" si="0"/>
+        <v>91</v>
+      </c>
+      <c r="H21" s="9">
+        <f t="shared" ca="1" si="0"/>
         <v>87</v>
       </c>
-      <c r="H21" s="9">
-        <f t="shared" ca="1" si="0"/>
-        <v>69</v>
-      </c>
       <c r="I21" s="9">
         <f t="shared" ca="1" si="1"/>
-        <v>55</v>
+        <v>49</v>
       </c>
       <c r="J21" s="9">
         <f t="shared" ca="1" si="1"/>
-        <v>41</v>
+        <v>33</v>
       </c>
       <c r="K21" s="8"/>
     </row>
@@ -2763,19 +2763,19 @@
       </c>
       <c r="G22" s="9">
         <f t="shared" ca="1" si="0"/>
-        <v>81</v>
+        <v>66</v>
       </c>
       <c r="H22" s="9">
         <f t="shared" ca="1" si="0"/>
-        <v>73</v>
+        <v>65</v>
       </c>
       <c r="I22" s="9">
         <f t="shared" ca="1" si="1"/>
-        <v>53</v>
+        <v>46</v>
       </c>
       <c r="J22" s="9">
         <f t="shared" ca="1" si="1"/>
-        <v>44</v>
+        <v>49</v>
       </c>
       <c r="K22" s="8"/>
     </row>
@@ -2800,19 +2800,19 @@
       </c>
       <c r="G23" s="9">
         <f t="shared" ca="1" si="0"/>
-        <v>60</v>
+        <v>68</v>
       </c>
       <c r="H23" s="9">
         <f t="shared" ca="1" si="0"/>
-        <v>66</v>
+        <v>69</v>
       </c>
       <c r="I23" s="9">
         <f t="shared" ca="1" si="1"/>
-        <v>51</v>
+        <v>47</v>
       </c>
       <c r="J23" s="9">
         <f t="shared" ca="1" si="1"/>
-        <v>34</v>
+        <v>40</v>
       </c>
       <c r="K23" s="8"/>
     </row>
@@ -2837,19 +2837,19 @@
       </c>
       <c r="G24" s="9">
         <f t="shared" ca="1" si="0"/>
-        <v>85</v>
+        <v>71</v>
       </c>
       <c r="H24" s="9">
         <f t="shared" ca="1" si="0"/>
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="I24" s="9">
         <f t="shared" ca="1" si="1"/>
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="J24" s="9">
         <f t="shared" ca="1" si="1"/>
-        <v>38</v>
+        <v>48</v>
       </c>
       <c r="K24" s="8"/>
     </row>
@@ -2874,11 +2874,11 @@
       </c>
       <c r="G25" s="9">
         <f t="shared" ca="1" si="0"/>
-        <v>75</v>
+        <v>71</v>
       </c>
       <c r="H25" s="9">
         <f t="shared" ca="1" si="0"/>
-        <v>87</v>
+        <v>74</v>
       </c>
       <c r="I25" s="9">
         <f t="shared" ca="1" si="1"/>
@@ -2886,7 +2886,7 @@
       </c>
       <c r="J25" s="9">
         <f t="shared" ca="1" si="1"/>
-        <v>32</v>
+        <v>57</v>
       </c>
       <c r="K25" s="8"/>
     </row>
@@ -2911,19 +2911,19 @@
       </c>
       <c r="G26" s="9">
         <f t="shared" ca="1" si="0"/>
-        <v>81</v>
+        <v>73</v>
       </c>
       <c r="H26" s="9">
         <f t="shared" ca="1" si="0"/>
-        <v>95</v>
+        <v>64</v>
       </c>
       <c r="I26" s="9">
         <f t="shared" ca="1" si="1"/>
-        <v>41</v>
+        <v>44</v>
       </c>
       <c r="J26" s="9">
         <f t="shared" ca="1" si="1"/>
-        <v>33</v>
+        <v>54</v>
       </c>
       <c r="K26" s="8"/>
     </row>
@@ -2948,19 +2948,19 @@
       </c>
       <c r="G27" s="9">
         <f t="shared" ca="1" si="0"/>
-        <v>77</v>
+        <v>61</v>
       </c>
       <c r="H27" s="9">
         <f t="shared" ca="1" si="0"/>
-        <v>98</v>
+        <v>63</v>
       </c>
       <c r="I27" s="9">
         <f t="shared" ca="1" si="1"/>
-        <v>51</v>
+        <v>35</v>
       </c>
       <c r="J27" s="9">
         <f t="shared" ca="1" si="1"/>
-        <v>39</v>
+        <v>50</v>
       </c>
       <c r="K27" s="8"/>
     </row>
@@ -2985,19 +2985,19 @@
       </c>
       <c r="G28" s="9">
         <f t="shared" ca="1" si="0"/>
-        <v>96</v>
+        <v>72</v>
       </c>
       <c r="H28" s="9">
         <f t="shared" ca="1" si="0"/>
-        <v>79</v>
+        <v>72</v>
       </c>
       <c r="I28" s="9">
         <f t="shared" ca="1" si="1"/>
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="J28" s="9">
         <f t="shared" ca="1" si="1"/>
-        <v>41</v>
+        <v>45</v>
       </c>
       <c r="K28" s="8"/>
     </row>
@@ -3022,19 +3022,19 @@
       </c>
       <c r="G29" s="9">
         <f t="shared" ca="1" si="0"/>
-        <v>84</v>
+        <v>68</v>
       </c>
       <c r="H29" s="9">
         <f t="shared" ca="1" si="0"/>
-        <v>88</v>
+        <v>76</v>
       </c>
       <c r="I29" s="9">
         <f t="shared" ca="1" si="1"/>
-        <v>31</v>
+        <v>48</v>
       </c>
       <c r="J29" s="9">
         <f t="shared" ca="1" si="1"/>
-        <v>41</v>
+        <v>46</v>
       </c>
       <c r="K29" s="8"/>
     </row>
@@ -3059,19 +3059,19 @@
       </c>
       <c r="G30" s="9">
         <f t="shared" ca="1" si="0"/>
-        <v>95</v>
+        <v>85</v>
       </c>
       <c r="H30" s="9">
         <f t="shared" ca="1" si="0"/>
-        <v>78</v>
+        <v>60</v>
       </c>
       <c r="I30" s="9">
         <f t="shared" ca="1" si="1"/>
-        <v>48</v>
+        <v>59</v>
       </c>
       <c r="J30" s="9">
         <f t="shared" ca="1" si="1"/>
-        <v>38</v>
+        <v>43</v>
       </c>
       <c r="K30" s="8"/>
     </row>
@@ -3096,19 +3096,19 @@
       </c>
       <c r="G31" s="9">
         <f t="shared" ca="1" si="0"/>
-        <v>79</v>
+        <v>68</v>
       </c>
       <c r="H31" s="9">
         <f t="shared" ca="1" si="0"/>
-        <v>63</v>
+        <v>68</v>
       </c>
       <c r="I31" s="9">
         <f t="shared" ca="1" si="1"/>
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="J31" s="9">
         <f t="shared" ca="1" si="1"/>
-        <v>48</v>
+        <v>31</v>
       </c>
       <c r="K31" s="8"/>
     </row>
@@ -3133,19 +3133,19 @@
       </c>
       <c r="G32" s="9">
         <f t="shared" ca="1" si="0"/>
-        <v>95</v>
+        <v>62</v>
       </c>
       <c r="H32" s="9">
         <f t="shared" ca="1" si="0"/>
-        <v>83</v>
+        <v>92</v>
       </c>
       <c r="I32" s="9">
         <f t="shared" ca="1" si="1"/>
-        <v>58</v>
+        <v>55</v>
       </c>
       <c r="J32" s="9">
         <f t="shared" ca="1" si="1"/>
-        <v>46</v>
+        <v>41</v>
       </c>
       <c r="K32" s="8"/>
     </row>
@@ -3170,19 +3170,19 @@
       </c>
       <c r="G33" s="9">
         <f t="shared" ca="1" si="0"/>
-        <v>90</v>
+        <v>96</v>
       </c>
       <c r="H33" s="9">
         <f t="shared" ca="1" si="0"/>
-        <v>99</v>
+        <v>93</v>
       </c>
       <c r="I33" s="9">
         <f t="shared" ca="1" si="1"/>
-        <v>42</v>
+        <v>48</v>
       </c>
       <c r="J33" s="9">
         <f t="shared" ca="1" si="1"/>
-        <v>46</v>
+        <v>54</v>
       </c>
       <c r="K33" s="8"/>
     </row>
@@ -3207,19 +3207,19 @@
       </c>
       <c r="G34" s="9">
         <f t="shared" ca="1" si="0"/>
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="H34" s="9">
         <f t="shared" ca="1" si="0"/>
-        <v>82</v>
+        <v>76</v>
       </c>
       <c r="I34" s="9">
         <f t="shared" ca="1" si="1"/>
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="J34" s="9">
         <f t="shared" ca="1" si="1"/>
-        <v>46</v>
+        <v>43</v>
       </c>
       <c r="K34" s="8"/>
     </row>
@@ -3244,19 +3244,19 @@
       </c>
       <c r="G35" s="9">
         <f t="shared" ca="1" si="0"/>
-        <v>60</v>
+        <v>73</v>
       </c>
       <c r="H35" s="9">
         <f t="shared" ca="1" si="0"/>
-        <v>82</v>
+        <v>62</v>
       </c>
       <c r="I35" s="9">
         <f t="shared" ca="1" si="1"/>
-        <v>37</v>
+        <v>44</v>
       </c>
       <c r="J35" s="9">
         <f t="shared" ca="1" si="1"/>
-        <v>39</v>
+        <v>57</v>
       </c>
       <c r="K35" s="8"/>
     </row>
@@ -3281,19 +3281,19 @@
       </c>
       <c r="G36" s="9">
         <f t="shared" ca="1" si="0"/>
-        <v>92</v>
+        <v>87</v>
       </c>
       <c r="H36" s="9">
         <f t="shared" ca="1" si="0"/>
-        <v>76</v>
+        <v>71</v>
       </c>
       <c r="I36" s="9">
         <f t="shared" ca="1" si="1"/>
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="J36" s="9">
         <f t="shared" ca="1" si="1"/>
-        <v>31</v>
+        <v>49</v>
       </c>
       <c r="K36" s="8"/>
     </row>
@@ -3318,19 +3318,19 @@
       </c>
       <c r="G37" s="9">
         <f t="shared" ca="1" si="0"/>
-        <v>76</v>
+        <v>89</v>
       </c>
       <c r="H37" s="9">
         <f t="shared" ca="1" si="0"/>
-        <v>78</v>
+        <v>63</v>
       </c>
       <c r="I37" s="9">
         <f t="shared" ca="1" si="1"/>
-        <v>39</v>
+        <v>31</v>
       </c>
       <c r="J37" s="9">
         <f t="shared" ca="1" si="1"/>
-        <v>59</v>
+        <v>53</v>
       </c>
       <c r="K37" s="8"/>
     </row>
@@ -3355,15 +3355,15 @@
       </c>
       <c r="G38" s="9">
         <f t="shared" ca="1" si="0"/>
-        <v>66</v>
+        <v>74</v>
       </c>
       <c r="H38" s="9">
         <f t="shared" ca="1" si="0"/>
-        <v>72</v>
+        <v>97</v>
       </c>
       <c r="I38" s="9">
         <f t="shared" ca="1" si="1"/>
-        <v>34</v>
+        <v>48</v>
       </c>
       <c r="J38" s="9">
         <f t="shared" ca="1" si="1"/>
@@ -3392,19 +3392,19 @@
       </c>
       <c r="G39" s="9">
         <f t="shared" ca="1" si="0"/>
-        <v>78</v>
+        <v>72</v>
       </c>
       <c r="H39" s="9">
         <f t="shared" ca="1" si="0"/>
-        <v>90</v>
+        <v>77</v>
       </c>
       <c r="I39" s="9">
         <f t="shared" ca="1" si="1"/>
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="J39" s="9">
         <f t="shared" ca="1" si="1"/>
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="K39" s="8"/>
     </row>
@@ -3429,19 +3429,19 @@
       </c>
       <c r="G40" s="9">
         <f t="shared" ca="1" si="0"/>
-        <v>85</v>
+        <v>98</v>
       </c>
       <c r="H40" s="9">
         <f t="shared" ca="1" si="0"/>
-        <v>77</v>
+        <v>68</v>
       </c>
       <c r="I40" s="9">
         <f t="shared" ca="1" si="1"/>
-        <v>34</v>
+        <v>47</v>
       </c>
       <c r="J40" s="9">
         <f t="shared" ca="1" si="1"/>
-        <v>33</v>
+        <v>39</v>
       </c>
       <c r="K40" s="8"/>
     </row>
@@ -3466,15 +3466,15 @@
       </c>
       <c r="G41" s="9">
         <f t="shared" ca="1" si="0"/>
-        <v>75</v>
+        <v>64</v>
       </c>
       <c r="H41" s="9">
         <f t="shared" ca="1" si="0"/>
-        <v>93</v>
+        <v>68</v>
       </c>
       <c r="I41" s="9">
         <f t="shared" ca="1" si="1"/>
-        <v>54</v>
+        <v>50</v>
       </c>
       <c r="J41" s="9">
         <f t="shared" ca="1" si="1"/>
@@ -3503,19 +3503,19 @@
       </c>
       <c r="G42" s="9">
         <f t="shared" ca="1" si="0"/>
-        <v>99</v>
+        <v>83</v>
       </c>
       <c r="H42" s="9">
         <f t="shared" ca="1" si="0"/>
-        <v>89</v>
+        <v>72</v>
       </c>
       <c r="I42" s="9">
         <f t="shared" ca="1" si="1"/>
-        <v>57</v>
+        <v>40</v>
       </c>
       <c r="J42" s="9">
         <f t="shared" ca="1" si="1"/>
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="K42" s="8"/>
     </row>
@@ -3540,19 +3540,19 @@
       </c>
       <c r="G43" s="9">
         <f t="shared" ca="1" si="0"/>
-        <v>80</v>
+        <v>83</v>
       </c>
       <c r="H43" s="9">
         <f t="shared" ca="1" si="0"/>
-        <v>95</v>
+        <v>98</v>
       </c>
       <c r="I43" s="9">
         <f t="shared" ca="1" si="1"/>
-        <v>59</v>
+        <v>39</v>
       </c>
       <c r="J43" s="9">
         <f t="shared" ca="1" si="1"/>
-        <v>37</v>
+        <v>31</v>
       </c>
       <c r="K43" s="8"/>
     </row>
@@ -3577,19 +3577,19 @@
       </c>
       <c r="G44" s="9">
         <f t="shared" ca="1" si="0"/>
-        <v>73</v>
+        <v>83</v>
       </c>
       <c r="H44" s="9">
         <f t="shared" ca="1" si="0"/>
-        <v>78</v>
+        <v>60</v>
       </c>
       <c r="I44" s="9">
         <f t="shared" ca="1" si="1"/>
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="J44" s="9">
         <f t="shared" ca="1" si="1"/>
-        <v>33</v>
+        <v>54</v>
       </c>
       <c r="K44" s="8"/>
     </row>
@@ -3614,19 +3614,19 @@
       </c>
       <c r="G45" s="9">
         <f t="shared" ca="1" si="0"/>
+        <v>68</v>
+      </c>
+      <c r="H45" s="9">
+        <f t="shared" ca="1" si="0"/>
         <v>89</v>
       </c>
-      <c r="H45" s="9">
-        <f t="shared" ca="1" si="0"/>
-        <v>75</v>
-      </c>
       <c r="I45" s="9">
         <f t="shared" ca="1" si="1"/>
-        <v>56</v>
+        <v>34</v>
       </c>
       <c r="J45" s="9">
         <f t="shared" ca="1" si="1"/>
-        <v>56</v>
+        <v>30</v>
       </c>
       <c r="K45" s="8"/>
     </row>
@@ -3651,19 +3651,19 @@
       </c>
       <c r="G46" s="9">
         <f t="shared" ca="1" si="0"/>
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="H46" s="9">
         <f t="shared" ca="1" si="0"/>
-        <v>99</v>
+        <v>81</v>
       </c>
       <c r="I46" s="9">
         <f t="shared" ca="1" si="1"/>
-        <v>45</v>
+        <v>35</v>
       </c>
       <c r="J46" s="9">
         <f t="shared" ca="1" si="1"/>
-        <v>53</v>
+        <v>34</v>
       </c>
       <c r="K46" s="8"/>
     </row>
@@ -3688,19 +3688,19 @@
       </c>
       <c r="G47" s="9">
         <f t="shared" ca="1" si="0"/>
-        <v>95</v>
+        <v>78</v>
       </c>
       <c r="H47" s="9">
         <f t="shared" ca="1" si="0"/>
-        <v>72</v>
+        <v>92</v>
       </c>
       <c r="I47" s="9">
         <f t="shared" ca="1" si="1"/>
-        <v>38</v>
+        <v>53</v>
       </c>
       <c r="J47" s="9">
         <f t="shared" ca="1" si="1"/>
-        <v>53</v>
+        <v>34</v>
       </c>
       <c r="K47" s="8"/>
     </row>
@@ -3725,19 +3725,19 @@
       </c>
       <c r="G48" s="9">
         <f t="shared" ca="1" si="0"/>
-        <v>94</v>
+        <v>70</v>
       </c>
       <c r="H48" s="9">
         <f t="shared" ca="1" si="0"/>
-        <v>93</v>
+        <v>89</v>
       </c>
       <c r="I48" s="9">
         <f t="shared" ca="1" si="1"/>
-        <v>53</v>
+        <v>58</v>
       </c>
       <c r="J48" s="9">
         <f t="shared" ca="1" si="1"/>
-        <v>45</v>
+        <v>57</v>
       </c>
       <c r="K48" s="8"/>
     </row>
@@ -3762,19 +3762,19 @@
       </c>
       <c r="G49" s="9">
         <f t="shared" ca="1" si="0"/>
-        <v>87</v>
+        <v>75</v>
       </c>
       <c r="H49" s="9">
         <f t="shared" ca="1" si="0"/>
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="I49" s="9">
         <f t="shared" ca="1" si="1"/>
-        <v>46</v>
+        <v>51</v>
       </c>
       <c r="J49" s="9">
         <f t="shared" ca="1" si="1"/>
-        <v>30</v>
+        <v>48</v>
       </c>
       <c r="K49" s="8"/>
     </row>
@@ -3799,19 +3799,19 @@
       </c>
       <c r="G50" s="9">
         <f t="shared" ca="1" si="0"/>
-        <v>61</v>
+        <v>72</v>
       </c>
       <c r="H50" s="9">
         <f t="shared" ca="1" si="0"/>
-        <v>74</v>
+        <v>84</v>
       </c>
       <c r="I50" s="9">
         <f t="shared" ca="1" si="1"/>
-        <v>45</v>
+        <v>54</v>
       </c>
       <c r="J50" s="9">
         <f t="shared" ca="1" si="1"/>
-        <v>32</v>
+        <v>40</v>
       </c>
       <c r="K50" s="8"/>
     </row>

</xml_diff>